<commit_message>
sankey to include multiR
</commit_message>
<xml_diff>
--- a/ReportDefs-KINESYS_Batt.xlsx
+++ b/ReportDefs-KINESYS_Batt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\KiNESYS_BattCircularity-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794C2BFD-54D1-43C5-82E3-670DF6164709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A5F121-1FDC-4185-9727-4142B3A4E963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="64" r:id="rId1"/>
@@ -11909,7 +11909,7 @@
     <t>~TS_Defs: Snk_attr=SANKEY_Battery</t>
   </si>
   <si>
-    <t>m_*,mr_*</t>
+    <t>m_*,mr_*,multir*</t>
   </si>
 </sst>
 </file>

</xml_diff>